<commit_message>
Add benchmark and testing scripts for genetic algorithm and Gurobi optimization
- Created benchmark.py and benchmark_instances.py for benchmarking purposes.
- Implemented dashboard_scenarios.py for scenario analysis with genetic algorithms.
- Added test scripts for genetic algorithm (testGA_small.py, test_ga_small.py) and Gurobi (test_gurobi.py, test_gurobi_compatibility.py, test_gurobi_linecompatibility.py, test_gurobi_operators.py).
- Introduced optimality gap test script (test_optimality_gap.py).
- Included a sample input file (Inputs_July.xlsx) for testing.
</commit_message>
<xml_diff>
--- a/Inputs_EmpresaXReal.xlsx
+++ b/Inputs_EmpresaXReal.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaizen\Documents\tese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B5D4D0-984B-4685-B133-00F76151EB1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F25ACB-714A-4512-90AE-9591ADD70C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_ESTRUTURA" sheetId="2" state="hidden" r:id="rId1"/>
     <sheet name="2_REFERENCIAS" sheetId="3" r:id="rId2"/>
     <sheet name="3_SETUPS" sheetId="5" r:id="rId3"/>
     <sheet name="5_PROCURA" sheetId="8" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="9" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -762,7 +763,7 @@
     <author>tc={C7364A66-A497-423F-B38F-AF51BEC19DB7}</author>
   </authors>
   <commentList>
-    <comment ref="J35" authorId="0" shapeId="0" xr:uid="{C7364A66-A497-423F-B38F-AF51BEC19DB7}">
+    <comment ref="J34" authorId="0" shapeId="0" xr:uid="{C7364A66-A497-423F-B38F-AF51BEC19DB7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -775,7 +776,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2149" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2428" uniqueCount="534">
   <si>
     <t>ESTRUTURA FÍSICA DO SISTEMA PRODUTIVO</t>
   </si>
@@ -2347,15 +2348,46 @@
   </si>
   <si>
     <t>DC102600</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>Segunda</t>
+  </si>
+  <si>
+    <t>Terça</t>
+  </si>
+  <si>
+    <t>Quarta</t>
+  </si>
+  <si>
+    <t>Quinta</t>
+  </si>
+  <si>
+    <t>Sexta</t>
+  </si>
+  <si>
+    <t>DC804600R</t>
+  </si>
+  <si>
+    <t>l1</t>
+  </si>
+  <si>
+    <t>l2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General\ &quot;min&quot;"/>
     <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="170" formatCode="dd\-mm\-yyyy;@"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -2648,7 +2680,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2793,25 +2825,25 @@
     <xf numFmtId="14" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2823,17 +2855,644 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="106">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFADBCA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FFEEEED2"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5DBF3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF47D359"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3574,26 +4233,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104" tableBorderDxfId="103">
   <autoFilter ref="A4:Q192" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="14"/>
-    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="1"/>
-    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="101"/>
+    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="100"/>
+    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="99"/>
+    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="98"/>
+    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="97"/>
+    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="96"/>
+    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="95"/>
+    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="94"/>
+    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="93"/>
+    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="92"/>
+    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="91"/>
+    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="90"/>
+    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="89"/>
+    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="88"/>
+    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="87"/>
+    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3884,7 +4543,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="J35" dT="2026-05-21T13:53:57.62" personId="{DAA1B03B-E46D-4B86-913A-0A7B4214C9B3}" id="{C7364A66-A497-423F-B38F-AF51BEC19DB7}">
+  <threadedComment ref="J34" dT="2026-05-21T13:53:57.62" personId="{DAA1B03B-E46D-4B86-913A-0A7B4214C9B3}" id="{C7364A66-A497-423F-B38F-AF51BEC19DB7}">
     <text>900</text>
   </threadedComment>
 </ThreadedComments>
@@ -3940,11 +4599,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -3976,7 +4635,7 @@
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="53" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="54"/>
@@ -4013,7 +4672,7 @@
       <c r="C9" s="3"/>
     </row>
     <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="57" t="s">
+      <c r="A11" s="53" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="54"/>
@@ -4041,7 +4700,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="57" t="s">
+      <c r="A15" s="53" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="54"/>
@@ -4127,7 +4786,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="53" t="s">
         <v>19</v>
       </c>
       <c r="B24" s="54"/>
@@ -4211,7 +4870,7 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="57" t="s">
+      <c r="A33" s="53" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="54"/>
@@ -4240,64 +4899,59 @@
       <c r="A39" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="56"/>
-      <c r="C39" s="56"/>
+      <c r="B39" s="57"/>
+      <c r="C39" s="57"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="56"/>
-      <c r="C40" s="56"/>
+      <c r="B40" s="57"/>
+      <c r="C40" s="57"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="59"/>
-      <c r="B41" s="56"/>
-      <c r="C41" s="56"/>
+      <c r="B41" s="57"/>
+      <c r="C41" s="57"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="56"/>
-      <c r="C42" s="56"/>
+      <c r="B42" s="57"/>
+      <c r="C42" s="57"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" s="55" t="s">
+      <c r="A43" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="56"/>
-      <c r="C43" s="56"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="57"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="B44" s="56"/>
-      <c r="C44" s="56"/>
+      <c r="B44" s="57"/>
+      <c r="C44" s="57"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" s="53"/>
+      <c r="A45" s="55"/>
       <c r="B45" s="54"/>
       <c r="C45" s="54"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="53"/>
+      <c r="A46" s="55"/>
       <c r="B46" s="54"/>
       <c r="C46" s="54"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" s="53"/>
+      <c r="A47" s="55"/>
       <c r="B47" s="54"/>
       <c r="C47" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A43:C43"/>
@@ -4309,6 +4963,11 @@
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A46:C46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4340,44 +4999,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
-      <c r="O1" s="51"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
+      <c r="N1" s="52"/>
+      <c r="O1" s="52"/>
     </row>
     <row r="2" spans="1:17" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="52"/>
-      <c r="L2" s="52"/>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
     </row>
     <row r="4" spans="1:17" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
@@ -14639,70 +15298,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
-      <c r="V1" s="51"/>
-      <c r="W1" s="51"/>
-      <c r="X1" s="51"/>
-      <c r="Y1" s="51"/>
-      <c r="Z1" s="51"/>
-      <c r="AA1" s="51"/>
-      <c r="AB1" s="51"/>
-      <c r="AC1" s="51"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
+      <c r="N1" s="52"/>
+      <c r="O1" s="52"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="52"/>
+      <c r="V1" s="52"/>
+      <c r="W1" s="52"/>
+      <c r="X1" s="52"/>
+      <c r="Y1" s="52"/>
+      <c r="Z1" s="52"/>
+      <c r="AA1" s="52"/>
+      <c r="AB1" s="52"/>
+      <c r="AC1" s="52"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="50" t="s">
         <v>400</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="M2" s="51"/>
-      <c r="N2" s="51"/>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
-      <c r="Q2" s="51"/>
-      <c r="R2" s="51"/>
-      <c r="S2" s="51"/>
-      <c r="T2" s="51"/>
-      <c r="U2" s="51"/>
-      <c r="V2" s="51"/>
-      <c r="W2" s="51"/>
-      <c r="X2" s="51"/>
-      <c r="Y2" s="51"/>
-      <c r="Z2" s="51"/>
-      <c r="AA2" s="51"/>
-      <c r="AB2" s="51"/>
-      <c r="AC2" s="51"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="52"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52"/>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="52"/>
+      <c r="AC2" s="52"/>
     </row>
     <row r="3" spans="1:38" ht="32" x14ac:dyDescent="0.7">
       <c r="B3" s="63" t="s">
@@ -18733,7 +19392,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="B1:J93"/>
+  <dimension ref="B1:J81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14" style="4" customWidth="1"/>
@@ -18746,1013 +19405,2790 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-    </row>
-    <row r="2" spans="2:4" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-    </row>
-    <row r="4" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B4" s="28" t="s">
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+    </row>
+    <row r="3" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C3" s="47" t="s">
         <v>404</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D3" s="29" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B4" s="46" t="s">
+        <v>255</v>
+      </c>
+      <c r="C4" s="46">
+        <v>120</v>
+      </c>
+      <c r="D4" s="49">
+        <v>46203</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" s="46" t="s">
-        <v>224</v>
+        <v>330</v>
       </c>
       <c r="C5" s="46">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="D5" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="46" t="s">
-        <v>372</v>
+        <v>389</v>
       </c>
       <c r="C6" s="46">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D6" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="46" t="s">
-        <v>521</v>
+        <v>328</v>
       </c>
       <c r="C7" s="46">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="D7" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="46" t="s">
-        <v>234</v>
+        <v>396</v>
       </c>
       <c r="C8" s="46">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D8" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="46" t="s">
-        <v>374</v>
+        <v>326</v>
       </c>
       <c r="C9" s="46">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D9" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B10" s="46" t="s">
-        <v>267</v>
+        <v>326</v>
       </c>
       <c r="C10" s="46">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="D10" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11" s="46" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="C11" s="46">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D11" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B12" s="46" t="s">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="C12" s="46">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="D12" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="46" t="s">
-        <v>322</v>
+        <v>389</v>
       </c>
       <c r="C13" s="46">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="D13" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B14" s="46" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C14" s="46">
-        <v>54</v>
+        <v>432</v>
       </c>
       <c r="D14" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B15" s="46" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C15" s="46">
-        <v>432</v>
+        <v>108</v>
       </c>
       <c r="D15" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B16" s="46" t="s">
-        <v>345</v>
+        <v>374</v>
       </c>
       <c r="C16" s="46">
         <v>108</v>
       </c>
       <c r="D16" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" s="46" t="s">
-        <v>349</v>
+        <v>269</v>
       </c>
       <c r="C17" s="46">
-        <v>108</v>
+        <v>42</v>
       </c>
       <c r="D17" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="46" t="s">
-        <v>385</v>
+        <v>333</v>
       </c>
       <c r="C18" s="46">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D18" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="46" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C19" s="46">
-        <v>54</v>
+        <v>800</v>
       </c>
       <c r="D19" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="46" t="s">
-        <v>242</v>
+        <v>270</v>
       </c>
       <c r="C20" s="46">
         <v>800</v>
       </c>
       <c r="D20" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="46" t="s">
-        <v>243</v>
+        <v>282</v>
       </c>
       <c r="C21" s="46">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="D21" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B22" s="46" t="s">
-        <v>244</v>
+        <v>365</v>
       </c>
       <c r="C22" s="46">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="D22" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B23" s="46" t="s">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="C23" s="46">
-        <v>116</v>
+        <v>48</v>
       </c>
       <c r="D23" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B24" s="46" t="s">
-        <v>246</v>
+        <v>293</v>
       </c>
       <c r="C24" s="46">
-        <v>48</v>
+        <v>144</v>
       </c>
       <c r="D24" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B25" s="46" t="s">
-        <v>252</v>
+        <v>291</v>
       </c>
       <c r="C25" s="46">
-        <v>144</v>
+        <v>48</v>
       </c>
       <c r="D25" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B26" s="46" t="s">
-        <v>249</v>
+        <v>390</v>
       </c>
       <c r="C26" s="46">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="D26" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B27" s="46" t="s">
-        <v>248</v>
+        <v>372</v>
       </c>
       <c r="C27" s="46">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D27" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B28" s="46" t="s">
-        <v>250</v>
+        <v>378</v>
       </c>
       <c r="C28" s="46">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="D28" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B29" s="46" t="s">
-        <v>251</v>
+        <v>341</v>
       </c>
       <c r="C29" s="46">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="D29" s="49">
-        <v>46233</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B30" s="46" t="s">
-        <v>517</v>
+        <v>254</v>
       </c>
       <c r="C30" s="46">
-        <v>96</v>
+        <v>200</v>
       </c>
       <c r="D30" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B31" s="46" t="s">
-        <v>279</v>
+        <v>376</v>
       </c>
       <c r="C31" s="46">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D31" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B32" s="46" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="C32" s="46">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="D32" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B33" s="46" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C33" s="46">
-        <v>120</v>
+        <v>72</v>
       </c>
       <c r="D33" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B34" s="46" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C34" s="46">
-        <v>72</v>
+        <v>200</v>
       </c>
       <c r="D34" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B35" s="46" t="s">
-        <v>391</v>
+        <v>225</v>
       </c>
       <c r="C35" s="46">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D35" s="49">
-        <v>46233</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B36" s="46" t="s">
-        <v>297</v>
+        <v>224</v>
       </c>
       <c r="C36" s="46">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="D36" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B37" s="46" t="s">
-        <v>300</v>
+        <v>226</v>
       </c>
       <c r="C37" s="46">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="D37" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B38" s="46" t="s">
-        <v>308</v>
+        <v>364</v>
       </c>
       <c r="C38" s="46">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="D38" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B39" s="46" t="s">
-        <v>310</v>
+        <v>376</v>
       </c>
       <c r="C39" s="46">
-        <v>120</v>
+        <v>48</v>
       </c>
       <c r="D39" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B40" s="46" t="s">
-        <v>311</v>
+        <v>223</v>
       </c>
       <c r="C40" s="46">
-        <v>48</v>
+        <v>128</v>
       </c>
       <c r="D40" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B41" s="46" t="s">
-        <v>509</v>
+        <v>372</v>
       </c>
       <c r="C41" s="46">
-        <v>128</v>
+        <v>156</v>
       </c>
       <c r="D41" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B42" s="46" t="s">
-        <v>312</v>
+        <v>242</v>
       </c>
       <c r="C42" s="46">
-        <v>156</v>
+        <v>60</v>
       </c>
       <c r="D42" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B43" s="46" t="s">
-        <v>327</v>
+        <v>352</v>
       </c>
       <c r="C43" s="46">
-        <v>60</v>
+        <v>144</v>
       </c>
       <c r="D43" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B44" s="46" t="s">
-        <v>358</v>
+        <v>336</v>
       </c>
       <c r="C44" s="46">
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="D44" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B45" s="46" t="s">
-        <v>359</v>
+        <v>279</v>
       </c>
       <c r="C45" s="46">
         <v>72</v>
       </c>
       <c r="D45" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B46" s="46" t="s">
-        <v>361</v>
+        <v>260</v>
       </c>
       <c r="C46" s="46">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="D46" s="49">
-        <v>46233</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B47" s="46" t="s">
-        <v>363</v>
+        <v>517</v>
       </c>
       <c r="C47" s="46">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="D47" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B48" s="46" t="s">
-        <v>280</v>
+        <v>308</v>
       </c>
       <c r="C48" s="46">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="D48" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B49" s="46" t="s">
-        <v>365</v>
+        <v>232</v>
       </c>
       <c r="C49" s="46">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="D49" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B50" s="46" t="s">
-        <v>366</v>
+        <v>245</v>
       </c>
       <c r="C50" s="46">
-        <v>44</v>
+        <v>176</v>
       </c>
       <c r="D50" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B51" s="46" t="s">
-        <v>367</v>
+        <v>245</v>
       </c>
       <c r="C51" s="46">
-        <v>176</v>
+        <v>44</v>
       </c>
       <c r="D51" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B52" s="46" t="s">
-        <v>368</v>
+        <v>242</v>
       </c>
       <c r="C52" s="46">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="D52" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B53" s="46" t="s">
-        <v>369</v>
+        <v>242</v>
       </c>
       <c r="C53" s="46">
+        <v>44</v>
+      </c>
+      <c r="D53" s="49">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B54" s="46" t="s">
+        <v>242</v>
+      </c>
+      <c r="C54" s="46">
+        <v>176</v>
+      </c>
+      <c r="D54" s="49">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B55" s="46" t="s">
+        <v>243</v>
+      </c>
+      <c r="C55" s="46">
         <v>88</v>
       </c>
-      <c r="D53" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B54" s="46" t="s">
-        <v>370</v>
-      </c>
-      <c r="C54" s="46">
-        <v>44</v>
-      </c>
-      <c r="D54" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="55" spans="2:4" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B55" s="46" t="s">
-        <v>371</v>
-      </c>
-      <c r="C55" s="46">
-        <v>176</v>
-      </c>
       <c r="D55" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B56" s="46" t="s">
-        <v>301</v>
+        <v>252</v>
       </c>
       <c r="C56" s="46">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D56" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B57" s="46" t="s">
-        <v>313</v>
+        <v>265</v>
       </c>
       <c r="C57" s="46">
-        <v>96</v>
+        <v>31</v>
       </c>
       <c r="D57" s="49">
-        <v>46233</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B58" s="46" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="C58" s="46">
-        <v>31</v>
+        <v>88</v>
       </c>
       <c r="D58" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B59" s="46" t="s">
-        <v>377</v>
+        <v>346</v>
       </c>
       <c r="C59" s="46">
-        <v>88</v>
+        <v>168</v>
       </c>
       <c r="D59" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B60" s="46" t="s">
-        <v>314</v>
+        <v>348</v>
       </c>
       <c r="C60" s="46">
-        <v>168</v>
+        <v>96</v>
       </c>
       <c r="D60" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B61" s="46" t="s">
-        <v>235</v>
+        <v>301</v>
       </c>
       <c r="C61" s="46">
         <v>96</v>
       </c>
       <c r="D61" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B62" s="46" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="C62" s="46">
         <v>96</v>
       </c>
       <c r="D62" s="49">
-        <v>46233</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B63" s="46" t="s">
-        <v>236</v>
+        <v>531</v>
       </c>
       <c r="C63" s="46">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="D63" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B64" s="46" t="s">
-        <v>241</v>
+        <v>510</v>
       </c>
       <c r="C64" s="46">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="D64" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B65" s="46" t="s">
-        <v>254</v>
+        <v>376</v>
       </c>
       <c r="C65" s="46">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D65" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B66" s="46" t="s">
-        <v>255</v>
+        <v>375</v>
       </c>
       <c r="C66" s="46">
-        <v>30</v>
+        <v>2232</v>
       </c>
       <c r="D66" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B67" s="46" t="s">
-        <v>260</v>
+        <v>374</v>
       </c>
       <c r="C67" s="46">
-        <v>2232</v>
+        <v>2225</v>
       </c>
       <c r="D67" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B68" s="46" t="s">
-        <v>376</v>
+        <v>253</v>
       </c>
       <c r="C68" s="46">
-        <v>2225</v>
+        <v>16</v>
       </c>
       <c r="D68" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B69" s="46" t="s">
-        <v>295</v>
+        <v>233</v>
       </c>
       <c r="C69" s="46">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D69" s="49">
-        <v>46233</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B70" s="46" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="C70" s="46">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="D70" s="49">
-        <v>46233</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B71" s="46" t="s">
-        <v>305</v>
+        <v>376</v>
       </c>
       <c r="C71" s="46">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="D71" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B72" s="46" t="s">
-        <v>261</v>
+        <v>322</v>
       </c>
       <c r="C72" s="46">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D72" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B73" s="46" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="C73" s="46">
-        <v>16</v>
+        <v>485</v>
       </c>
       <c r="D73" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B74" s="46" t="s">
-        <v>352</v>
+        <v>510</v>
       </c>
       <c r="C74" s="46">
-        <v>485</v>
+        <v>53</v>
       </c>
       <c r="D74" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B75" s="46" t="s">
-        <v>341</v>
+        <v>298</v>
       </c>
       <c r="C75" s="46">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D75" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B76" s="46" t="s">
-        <v>362</v>
+        <v>328</v>
       </c>
       <c r="C76" s="46">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="D76" s="49">
-        <v>46233</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B77" s="46" t="s">
-        <v>360</v>
+        <v>327</v>
       </c>
       <c r="C77" s="46">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="D77" s="49">
-        <v>46233</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B78" s="46" t="s">
-        <v>321</v>
+        <v>261</v>
       </c>
       <c r="C78" s="46">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D78" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B79" s="46" t="s">
-        <v>375</v>
+        <v>297</v>
       </c>
       <c r="C79" s="46">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="D79" s="49">
-        <v>46233</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B80" s="46" t="s">
-        <v>258</v>
+        <v>362</v>
       </c>
       <c r="C80" s="46">
-        <v>126</v>
+        <v>54</v>
       </c>
       <c r="D80" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B81" s="46" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="C81" s="46">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="D81" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B82" s="46" t="s">
-        <v>339</v>
-      </c>
-      <c r="C82" s="46">
-        <v>109</v>
-      </c>
-      <c r="D82" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="83" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B83" s="46" t="s">
-        <v>325</v>
-      </c>
-      <c r="C83" s="46">
-        <v>1536</v>
-      </c>
-      <c r="D83" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="84" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B84" s="46" t="s">
-        <v>326</v>
-      </c>
-      <c r="C84" s="46">
-        <v>128</v>
-      </c>
-      <c r="D84" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="85" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B85" s="46" t="s">
-        <v>296</v>
-      </c>
-      <c r="C85" s="46">
-        <v>192</v>
-      </c>
-      <c r="D85" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="86" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B86" s="46" t="s">
-        <v>329</v>
-      </c>
-      <c r="C86" s="46">
-        <v>128</v>
-      </c>
-      <c r="D86" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="87" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B87" s="46" t="s">
-        <v>221</v>
-      </c>
-      <c r="C87" s="46">
-        <v>264</v>
-      </c>
-      <c r="D87" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="88" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B88" s="46" t="s">
-        <v>222</v>
-      </c>
-      <c r="C88" s="46">
-        <v>120</v>
-      </c>
-      <c r="D88" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="89" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B89" s="46" t="s">
-        <v>223</v>
-      </c>
-      <c r="C89" s="46">
-        <v>264</v>
-      </c>
-      <c r="D89" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="90" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B90" s="46" t="s">
-        <v>330</v>
-      </c>
-      <c r="C90" s="46">
-        <v>112</v>
-      </c>
-      <c r="D90" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="91" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B91" s="46" t="s">
-        <v>523</v>
-      </c>
-      <c r="C91" s="46">
-        <v>360</v>
-      </c>
-      <c r="D91" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="92" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B92" s="46" t="s">
-        <v>510</v>
-      </c>
-      <c r="C92" s="46">
-        <v>126</v>
-      </c>
-      <c r="D92" s="49">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="93" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B93" s="46" t="s">
-        <v>511</v>
-      </c>
-      <c r="C93" s="46">
-        <v>126</v>
-      </c>
-      <c r="D93" s="49">
-        <v>46233</v>
+        <v>46203</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:D2"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D5915C-7F5B-45E3-B980-62686FF8BD4A}">
+  <dimension ref="B3:K74"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.7265625" style="64" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" style="12"/>
+    <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B3" s="64">
+        <v>46174</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3">
+        <v>200</v>
+      </c>
+      <c r="G3">
+        <v>6000</v>
+      </c>
+      <c r="H3" t="s">
+        <v>524</v>
+      </c>
+      <c r="I3">
+        <v>7.6923076923076925</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>532</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B4" s="64">
+        <v>46175</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F4">
+        <v>112</v>
+      </c>
+      <c r="G4">
+        <v>112</v>
+      </c>
+      <c r="H4" t="s">
+        <v>524</v>
+      </c>
+      <c r="I4">
+        <v>0.62222222222222223</v>
+      </c>
+      <c r="J4" s="12">
+        <f>SUMIFS(I3:I74,H3:H74,"L1")</f>
+        <v>117.53216698351397</v>
+      </c>
+      <c r="K4" s="12">
+        <f>SUMIFS(I3:I74,H3:H74,"L2")</f>
+        <v>62.835831529581526</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B5" s="64">
+        <v>46175</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5">
+        <v>256</v>
+      </c>
+      <c r="G5">
+        <v>256</v>
+      </c>
+      <c r="H5" t="s">
+        <v>524</v>
+      </c>
+      <c r="I5">
+        <v>1.024</v>
+      </c>
+      <c r="J5">
+        <f>7.5*18</f>
+        <v>135</v>
+      </c>
+      <c r="K5">
+        <f>7.5*18</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B6" s="64">
+        <v>46175</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D6" t="s">
+        <v>328</v>
+      </c>
+      <c r="E6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6">
+        <v>64</v>
+      </c>
+      <c r="G6">
+        <v>256</v>
+      </c>
+      <c r="H6" t="s">
+        <v>524</v>
+      </c>
+      <c r="I6">
+        <v>1.024</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B7" s="64">
+        <v>46175</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D7" t="s">
+        <v>396</v>
+      </c>
+      <c r="E7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F7">
+        <v>512</v>
+      </c>
+      <c r="G7">
+        <v>512</v>
+      </c>
+      <c r="H7" t="s">
+        <v>524</v>
+      </c>
+      <c r="I7">
+        <v>2.8444444444444446</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B8" s="64">
+        <v>46175</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8">
+        <v>350</v>
+      </c>
+      <c r="G8">
+        <v>350</v>
+      </c>
+      <c r="H8" t="s">
+        <v>524</v>
+      </c>
+      <c r="I8">
+        <v>1.9444444444444444</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B9" s="64">
+        <v>46175</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D9" t="s">
+        <v>326</v>
+      </c>
+      <c r="E9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F9">
+        <v>128</v>
+      </c>
+      <c r="G9">
+        <v>128</v>
+      </c>
+      <c r="H9" t="s">
+        <v>524</v>
+      </c>
+      <c r="I9">
+        <v>0.71111111111111114</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B10" s="64">
+        <v>46176</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D10" t="s">
+        <v>259</v>
+      </c>
+      <c r="E10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10">
+        <v>200</v>
+      </c>
+      <c r="G10">
+        <v>400</v>
+      </c>
+      <c r="H10" t="s">
+        <v>524</v>
+      </c>
+      <c r="I10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B11" s="64">
+        <v>46176</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D11" t="s">
+        <v>329</v>
+      </c>
+      <c r="E11" t="s">
+        <v>153</v>
+      </c>
+      <c r="F11">
+        <v>256</v>
+      </c>
+      <c r="G11">
+        <v>256</v>
+      </c>
+      <c r="H11" t="s">
+        <v>524</v>
+      </c>
+      <c r="I11">
+        <v>1.024</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B12" s="64">
+        <v>46176</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D12" t="s">
+        <v>389</v>
+      </c>
+      <c r="E12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F12">
+        <v>256</v>
+      </c>
+      <c r="G12">
+        <v>256</v>
+      </c>
+      <c r="H12" t="s">
+        <v>524</v>
+      </c>
+      <c r="I12">
+        <v>1.024</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B13" s="64">
+        <v>46176</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D13" t="s">
+        <v>325</v>
+      </c>
+      <c r="E13" t="s">
+        <v>149</v>
+      </c>
+      <c r="F13">
+        <v>1280</v>
+      </c>
+      <c r="G13">
+        <v>1280</v>
+      </c>
+      <c r="H13" t="s">
+        <v>524</v>
+      </c>
+      <c r="I13">
+        <v>5.12</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B14" s="64">
+        <v>46176</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D14" t="s">
+        <v>375</v>
+      </c>
+      <c r="E14" t="s">
+        <v>199</v>
+      </c>
+      <c r="F14">
+        <v>128</v>
+      </c>
+      <c r="G14">
+        <v>3840</v>
+      </c>
+      <c r="H14" t="s">
+        <v>525</v>
+      </c>
+      <c r="I14">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B15" s="64">
+        <v>46176</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D15" t="s">
+        <v>374</v>
+      </c>
+      <c r="E15" t="s">
+        <v>198</v>
+      </c>
+      <c r="F15">
+        <v>128</v>
+      </c>
+      <c r="G15">
+        <v>3840</v>
+      </c>
+      <c r="H15" t="s">
+        <v>525</v>
+      </c>
+      <c r="I15">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B16" s="64">
+        <v>46181</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D16" t="s">
+        <v>269</v>
+      </c>
+      <c r="E16" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16">
+        <v>240</v>
+      </c>
+      <c r="G16">
+        <v>480</v>
+      </c>
+      <c r="H16" t="s">
+        <v>524</v>
+      </c>
+      <c r="I16">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B17" s="64">
+        <v>46181</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D17" t="s">
+        <v>333</v>
+      </c>
+      <c r="E17" t="s">
+        <v>157</v>
+      </c>
+      <c r="F17">
+        <v>63</v>
+      </c>
+      <c r="G17">
+        <v>252</v>
+      </c>
+      <c r="H17" t="s">
+        <v>524</v>
+      </c>
+      <c r="I17">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B18" s="64">
+        <v>46181</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D18" t="s">
+        <v>354</v>
+      </c>
+      <c r="E18" t="s">
+        <v>178</v>
+      </c>
+      <c r="F18">
+        <v>108</v>
+      </c>
+      <c r="G18">
+        <v>2268</v>
+      </c>
+      <c r="H18" t="s">
+        <v>524</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B19" s="64">
+        <v>46181</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E19" t="s">
+        <v>93</v>
+      </c>
+      <c r="F19">
+        <v>72</v>
+      </c>
+      <c r="G19">
+        <v>216</v>
+      </c>
+      <c r="H19" t="s">
+        <v>524</v>
+      </c>
+      <c r="I19">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B20" s="64">
+        <v>46181</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D20" t="s">
+        <v>282</v>
+      </c>
+      <c r="E20" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20">
+        <v>63</v>
+      </c>
+      <c r="G20">
+        <v>252</v>
+      </c>
+      <c r="H20" t="s">
+        <v>524</v>
+      </c>
+      <c r="I20">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B21" s="64">
+        <v>46181</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D21" t="s">
+        <v>365</v>
+      </c>
+      <c r="E21" t="s">
+        <v>189</v>
+      </c>
+      <c r="F21">
+        <v>176</v>
+      </c>
+      <c r="G21">
+        <v>352</v>
+      </c>
+      <c r="H21" t="s">
+        <v>524</v>
+      </c>
+      <c r="I21">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B22" s="64">
+        <v>46182</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D22" t="s">
+        <v>296</v>
+      </c>
+      <c r="E22" t="s">
+        <v>120</v>
+      </c>
+      <c r="F22">
+        <v>896</v>
+      </c>
+      <c r="G22">
+        <v>896</v>
+      </c>
+      <c r="H22" t="s">
+        <v>524</v>
+      </c>
+      <c r="I22">
+        <v>4.0727272727272723</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B23" s="64">
+        <v>46182</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D23" t="s">
+        <v>293</v>
+      </c>
+      <c r="E23" t="s">
+        <v>116</v>
+      </c>
+      <c r="F23">
+        <v>126</v>
+      </c>
+      <c r="G23">
+        <v>504</v>
+      </c>
+      <c r="H23" t="s">
+        <v>524</v>
+      </c>
+      <c r="I23">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B24" s="64">
+        <v>46182</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D24" t="s">
+        <v>291</v>
+      </c>
+      <c r="E24" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24">
+        <v>120</v>
+      </c>
+      <c r="G24">
+        <v>240</v>
+      </c>
+      <c r="H24" t="s">
+        <v>524</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B25" s="64">
+        <v>46182</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D25" t="s">
+        <v>390</v>
+      </c>
+      <c r="E25" t="s">
+        <v>214</v>
+      </c>
+      <c r="F25">
+        <v>156</v>
+      </c>
+      <c r="G25">
+        <v>312</v>
+      </c>
+      <c r="H25" t="s">
+        <v>524</v>
+      </c>
+      <c r="I25">
+        <v>2.3283582089552239</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B26" s="64">
+        <v>46182</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D26" t="s">
+        <v>372</v>
+      </c>
+      <c r="E26" t="s">
+        <v>196</v>
+      </c>
+      <c r="F26">
+        <v>144</v>
+      </c>
+      <c r="G26">
+        <v>6912</v>
+      </c>
+      <c r="H26" t="s">
+        <v>525</v>
+      </c>
+      <c r="I26">
+        <v>3.7894736842105261</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B27" s="64">
+        <v>46184</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D27" t="s">
+        <v>378</v>
+      </c>
+      <c r="E27" t="s">
+        <v>202</v>
+      </c>
+      <c r="F27">
+        <v>432</v>
+      </c>
+      <c r="G27">
+        <v>9072</v>
+      </c>
+      <c r="H27" t="s">
+        <v>524</v>
+      </c>
+      <c r="I27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B28" s="64">
+        <v>46184</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D28" t="s">
+        <v>341</v>
+      </c>
+      <c r="E28" t="s">
+        <v>165</v>
+      </c>
+      <c r="F28">
+        <v>216</v>
+      </c>
+      <c r="G28">
+        <v>4536</v>
+      </c>
+      <c r="H28" t="s">
+        <v>524</v>
+      </c>
+      <c r="I28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B29" s="64">
+        <v>46184</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D29" t="s">
+        <v>254</v>
+      </c>
+      <c r="E29" t="s">
+        <v>77</v>
+      </c>
+      <c r="F29">
+        <v>63</v>
+      </c>
+      <c r="G29">
+        <v>252</v>
+      </c>
+      <c r="H29" t="s">
+        <v>524</v>
+      </c>
+      <c r="I29">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B30" s="64">
+        <v>46184</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D30" t="s">
+        <v>376</v>
+      </c>
+      <c r="E30" t="s">
+        <v>200</v>
+      </c>
+      <c r="F30">
+        <v>306</v>
+      </c>
+      <c r="G30">
+        <v>7344</v>
+      </c>
+      <c r="H30" t="s">
+        <v>525</v>
+      </c>
+      <c r="I30">
+        <v>4.0263157894736841</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B31" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D31" t="s">
+        <v>298</v>
+      </c>
+      <c r="E31" t="s">
+        <v>122</v>
+      </c>
+      <c r="F31">
+        <v>48</v>
+      </c>
+      <c r="G31">
+        <v>192</v>
+      </c>
+      <c r="H31" t="s">
+        <v>524</v>
+      </c>
+      <c r="I31">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B32" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D32" t="s">
+        <v>287</v>
+      </c>
+      <c r="E32" t="s">
+        <v>110</v>
+      </c>
+      <c r="F32">
+        <v>96</v>
+      </c>
+      <c r="G32">
+        <v>384</v>
+      </c>
+      <c r="H32" t="s">
+        <v>524</v>
+      </c>
+      <c r="I32">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B33" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D33" t="s">
+        <v>288</v>
+      </c>
+      <c r="E33" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33">
+        <v>48</v>
+      </c>
+      <c r="G33">
+        <v>192</v>
+      </c>
+      <c r="H33" t="s">
+        <v>524</v>
+      </c>
+      <c r="I33">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B34" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D34" t="s">
+        <v>225</v>
+      </c>
+      <c r="E34" t="s">
+        <v>49</v>
+      </c>
+      <c r="F34">
+        <v>84</v>
+      </c>
+      <c r="G34">
+        <v>168</v>
+      </c>
+      <c r="H34" t="s">
+        <v>524</v>
+      </c>
+      <c r="I34">
+        <v>0.93333333333333335</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B35" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D35" t="s">
+        <v>224</v>
+      </c>
+      <c r="E35" t="s">
+        <v>48</v>
+      </c>
+      <c r="F35">
+        <v>84</v>
+      </c>
+      <c r="G35">
+        <v>168</v>
+      </c>
+      <c r="H35" t="s">
+        <v>524</v>
+      </c>
+      <c r="I35">
+        <v>0.93333333333333335</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B36" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D36" t="s">
+        <v>226</v>
+      </c>
+      <c r="E36" t="s">
+        <v>50</v>
+      </c>
+      <c r="F36">
+        <v>84</v>
+      </c>
+      <c r="G36">
+        <v>168</v>
+      </c>
+      <c r="H36" t="s">
+        <v>524</v>
+      </c>
+      <c r="I36">
+        <v>0.93333333333333335</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B37" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D37" t="s">
+        <v>364</v>
+      </c>
+      <c r="E37" t="s">
+        <v>188</v>
+      </c>
+      <c r="F37">
+        <v>72</v>
+      </c>
+      <c r="G37">
+        <v>216</v>
+      </c>
+      <c r="H37" t="s">
+        <v>525</v>
+      </c>
+      <c r="I37">
+        <v>0.98181818181818181</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B38" s="64">
+        <v>46185</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D38" t="s">
+        <v>376</v>
+      </c>
+      <c r="E38" t="s">
+        <v>200</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38" t="s">
+        <v>525</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B39" s="64">
+        <v>46189</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D39" t="s">
+        <v>352</v>
+      </c>
+      <c r="E39" t="s">
+        <v>176</v>
+      </c>
+      <c r="F39">
+        <v>480</v>
+      </c>
+      <c r="G39">
+        <v>480</v>
+      </c>
+      <c r="H39" t="s">
+        <v>524</v>
+      </c>
+      <c r="I39">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B40" s="64">
+        <v>46189</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D40" t="s">
+        <v>336</v>
+      </c>
+      <c r="E40" t="s">
+        <v>160</v>
+      </c>
+      <c r="F40">
+        <v>108</v>
+      </c>
+      <c r="G40">
+        <v>2268</v>
+      </c>
+      <c r="H40" t="s">
+        <v>524</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B41" s="64">
+        <v>46189</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D41" t="s">
+        <v>279</v>
+      </c>
+      <c r="E41" t="s">
+        <v>102</v>
+      </c>
+      <c r="F41">
+        <v>200</v>
+      </c>
+      <c r="G41">
+        <v>400</v>
+      </c>
+      <c r="H41" t="s">
+        <v>524</v>
+      </c>
+      <c r="I41">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B42" s="64">
+        <v>46190</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D42" t="s">
+        <v>260</v>
+      </c>
+      <c r="E42" t="s">
+        <v>83</v>
+      </c>
+      <c r="F42">
+        <v>432</v>
+      </c>
+      <c r="G42">
+        <v>1728</v>
+      </c>
+      <c r="H42" t="s">
+        <v>524</v>
+      </c>
+      <c r="I42">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B43" s="64">
+        <v>46190</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D43" t="s">
+        <v>517</v>
+      </c>
+      <c r="E43" t="s">
+        <v>516</v>
+      </c>
+      <c r="F43">
+        <v>192</v>
+      </c>
+      <c r="G43">
+        <v>384</v>
+      </c>
+      <c r="H43" t="s">
+        <v>525</v>
+      </c>
+      <c r="I43">
+        <v>3.0476190476190474</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B44" s="64">
+        <v>46191</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D44" t="s">
+        <v>308</v>
+      </c>
+      <c r="E44" t="s">
+        <v>132</v>
+      </c>
+      <c r="F44">
+        <v>192</v>
+      </c>
+      <c r="G44">
+        <v>384</v>
+      </c>
+      <c r="H44" t="s">
+        <v>525</v>
+      </c>
+      <c r="I44">
+        <v>3.0476190476190474</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B45" s="64">
+        <v>46191</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D45" t="s">
+        <v>232</v>
+      </c>
+      <c r="E45" t="s">
+        <v>56</v>
+      </c>
+      <c r="F45">
+        <v>140</v>
+      </c>
+      <c r="G45">
+        <v>6300</v>
+      </c>
+      <c r="H45" t="s">
+        <v>525</v>
+      </c>
+      <c r="I45">
+        <v>7.875</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B46" s="64">
+        <v>46191</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D46" t="s">
+        <v>245</v>
+      </c>
+      <c r="E46" t="s">
+        <v>68</v>
+      </c>
+      <c r="F46">
+        <v>88</v>
+      </c>
+      <c r="G46">
+        <v>7920</v>
+      </c>
+      <c r="H46" t="s">
+        <v>524</v>
+      </c>
+      <c r="I46">
+        <v>2.2916666666666665</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B47" s="64">
+        <v>46191</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D47" t="s">
+        <v>245</v>
+      </c>
+      <c r="E47" t="s">
+        <v>68</v>
+      </c>
+      <c r="F47">
+        <v>88</v>
+      </c>
+      <c r="G47">
+        <v>7920</v>
+      </c>
+      <c r="H47" t="s">
+        <v>525</v>
+      </c>
+      <c r="I47">
+        <v>2.2916666666666665</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B48" s="64">
+        <v>46192</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D48" t="s">
+        <v>242</v>
+      </c>
+      <c r="E48" t="s">
+        <v>65</v>
+      </c>
+      <c r="F48">
+        <v>250</v>
+      </c>
+      <c r="G48">
+        <v>22500</v>
+      </c>
+      <c r="H48" t="s">
+        <v>525</v>
+      </c>
+      <c r="I48">
+        <v>6.510416666666667</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B49" s="64">
+        <v>46192</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D49" t="s">
+        <v>242</v>
+      </c>
+      <c r="E49" t="s">
+        <v>65</v>
+      </c>
+      <c r="F49">
+        <v>250</v>
+      </c>
+      <c r="G49">
+        <v>22500</v>
+      </c>
+      <c r="H49" t="s">
+        <v>524</v>
+      </c>
+      <c r="I49">
+        <v>6.510416666666667</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B50" s="64">
+        <v>46195</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D50" t="s">
+        <v>243</v>
+      </c>
+      <c r="E50" t="s">
+        <v>66</v>
+      </c>
+      <c r="F50">
+        <v>300</v>
+      </c>
+      <c r="G50">
+        <v>27000</v>
+      </c>
+      <c r="H50" t="s">
+        <v>524</v>
+      </c>
+      <c r="I50">
+        <v>7.8125</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B51" s="64">
+        <v>46195</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D51" t="s">
+        <v>252</v>
+      </c>
+      <c r="E51" t="s">
+        <v>75</v>
+      </c>
+      <c r="F51">
+        <v>144</v>
+      </c>
+      <c r="G51">
+        <v>8208</v>
+      </c>
+      <c r="H51" t="s">
+        <v>525</v>
+      </c>
+      <c r="I51">
+        <v>3.5625</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B52" s="64">
+        <v>46195</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D52" t="s">
+        <v>265</v>
+      </c>
+      <c r="E52" t="s">
+        <v>88</v>
+      </c>
+      <c r="F52">
+        <v>256</v>
+      </c>
+      <c r="G52">
+        <v>256</v>
+      </c>
+      <c r="H52" t="s">
+        <v>525</v>
+      </c>
+      <c r="I52">
+        <v>4.2666666666666666</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B53" s="64">
+        <v>46196</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D53" t="s">
+        <v>260</v>
+      </c>
+      <c r="E53" t="s">
+        <v>83</v>
+      </c>
+      <c r="F53">
+        <v>432</v>
+      </c>
+      <c r="G53">
+        <v>1728</v>
+      </c>
+      <c r="H53" t="s">
+        <v>524</v>
+      </c>
+      <c r="I53">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B54" s="64">
+        <v>46197</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D54" t="s">
+        <v>346</v>
+      </c>
+      <c r="E54" t="s">
+        <v>170</v>
+      </c>
+      <c r="F54">
+        <v>108</v>
+      </c>
+      <c r="G54">
+        <v>2268</v>
+      </c>
+      <c r="H54" t="s">
+        <v>524</v>
+      </c>
+      <c r="I54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B55" s="64">
+        <v>46197</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D55" t="s">
+        <v>348</v>
+      </c>
+      <c r="E55" t="s">
+        <v>172</v>
+      </c>
+      <c r="F55">
+        <v>108</v>
+      </c>
+      <c r="G55">
+        <v>2268</v>
+      </c>
+      <c r="H55" t="s">
+        <v>524</v>
+      </c>
+      <c r="I55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B56" s="64">
+        <v>46197</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D56" t="s">
+        <v>301</v>
+      </c>
+      <c r="E56" t="s">
+        <v>125</v>
+      </c>
+      <c r="F56">
+        <v>176</v>
+      </c>
+      <c r="G56">
+        <v>352</v>
+      </c>
+      <c r="H56" t="s">
+        <v>524</v>
+      </c>
+      <c r="I56">
+        <v>1.9555555555555555</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B57" s="64">
+        <v>46197</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D57" t="s">
+        <v>300</v>
+      </c>
+      <c r="E57" t="s">
+        <v>124</v>
+      </c>
+      <c r="F57">
+        <v>240</v>
+      </c>
+      <c r="G57">
+        <v>480</v>
+      </c>
+      <c r="H57" t="s">
+        <v>525</v>
+      </c>
+      <c r="I57">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B58" s="64">
+        <v>46198</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D58" t="s">
+        <v>531</v>
+      </c>
+      <c r="E58" t="s">
+        <v>513</v>
+      </c>
+      <c r="F58">
+        <v>378</v>
+      </c>
+      <c r="G58">
+        <v>1512</v>
+      </c>
+      <c r="H58" t="s">
+        <v>524</v>
+      </c>
+      <c r="I58">
+        <v>4.32</v>
+      </c>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B59" s="64">
+        <v>46198</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D59" t="s">
+        <v>510</v>
+      </c>
+      <c r="E59" t="s">
+        <v>512</v>
+      </c>
+      <c r="F59">
+        <v>315</v>
+      </c>
+      <c r="G59">
+        <v>1260</v>
+      </c>
+      <c r="H59" t="s">
+        <v>524</v>
+      </c>
+      <c r="I59">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B60" s="64">
+        <v>46198</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D60" t="s">
+        <v>376</v>
+      </c>
+      <c r="E60" t="s">
+        <v>200</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60" t="s">
+        <v>525</v>
+      </c>
+      <c r="I60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B61" s="64">
+        <v>46198</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D61" t="s">
+        <v>375</v>
+      </c>
+      <c r="E61" t="s">
+        <v>199</v>
+      </c>
+      <c r="F61">
+        <v>128</v>
+      </c>
+      <c r="G61">
+        <v>3840</v>
+      </c>
+      <c r="H61" t="s">
+        <v>525</v>
+      </c>
+      <c r="I61">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B62" s="64">
+        <v>46198</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="D62" t="s">
+        <v>374</v>
+      </c>
+      <c r="E62" t="s">
+        <v>198</v>
+      </c>
+      <c r="F62">
+        <v>128</v>
+      </c>
+      <c r="G62">
+        <v>3840</v>
+      </c>
+      <c r="H62" t="s">
+        <v>525</v>
+      </c>
+      <c r="I62">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B63" s="64">
+        <v>46199</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D63" t="s">
+        <v>253</v>
+      </c>
+      <c r="E63" t="s">
+        <v>76</v>
+      </c>
+      <c r="F63">
+        <v>63</v>
+      </c>
+      <c r="G63">
+        <v>252</v>
+      </c>
+      <c r="H63" t="s">
+        <v>524</v>
+      </c>
+      <c r="I63">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="64" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B64" s="64">
+        <v>46199</v>
+      </c>
+      <c r="C64" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D64" t="s">
+        <v>233</v>
+      </c>
+      <c r="E64" t="s">
+        <v>57</v>
+      </c>
+      <c r="F64">
+        <v>140</v>
+      </c>
+      <c r="G64">
+        <v>5040</v>
+      </c>
+      <c r="H64" t="s">
+        <v>525</v>
+      </c>
+      <c r="I64">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="65" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B65" s="64">
+        <v>46199</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D65" t="s">
+        <v>311</v>
+      </c>
+      <c r="E65" t="s">
+        <v>135</v>
+      </c>
+      <c r="F65">
+        <v>96</v>
+      </c>
+      <c r="G65">
+        <v>192</v>
+      </c>
+      <c r="H65" t="s">
+        <v>524</v>
+      </c>
+      <c r="I65">
+        <v>1.5238095238095237</v>
+      </c>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B66" s="64">
+        <v>46199</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D66" t="s">
+        <v>376</v>
+      </c>
+      <c r="E66" t="s">
+        <v>200</v>
+      </c>
+      <c r="F66">
+        <v>204</v>
+      </c>
+      <c r="G66">
+        <v>4896</v>
+      </c>
+      <c r="H66" t="s">
+        <v>525</v>
+      </c>
+      <c r="I66">
+        <v>2.6842105263157894</v>
+      </c>
+    </row>
+    <row r="67" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B67" s="64">
+        <v>46202</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D67" t="s">
+        <v>510</v>
+      </c>
+      <c r="E67" t="s">
+        <v>512</v>
+      </c>
+      <c r="F67">
+        <v>11</v>
+      </c>
+      <c r="G67">
+        <v>44</v>
+      </c>
+      <c r="H67" t="s">
+        <v>524</v>
+      </c>
+      <c r="I67">
+        <v>0.12571428571428572</v>
+      </c>
+    </row>
+    <row r="68" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B68" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D68" t="s">
+        <v>298</v>
+      </c>
+      <c r="E68" t="s">
+        <v>122</v>
+      </c>
+      <c r="F68">
+        <v>48</v>
+      </c>
+      <c r="G68">
+        <v>192</v>
+      </c>
+      <c r="H68" t="s">
+        <v>524</v>
+      </c>
+      <c r="I68">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="69" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B69" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D69" t="s">
+        <v>328</v>
+      </c>
+      <c r="E69" t="s">
+        <v>152</v>
+      </c>
+      <c r="F69">
+        <v>32</v>
+      </c>
+      <c r="G69">
+        <v>128</v>
+      </c>
+      <c r="H69" t="s">
+        <v>524</v>
+      </c>
+      <c r="I69">
+        <v>0.51200000000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B70" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D70" t="s">
+        <v>327</v>
+      </c>
+      <c r="E70" t="s">
+        <v>151</v>
+      </c>
+      <c r="F70">
+        <v>120</v>
+      </c>
+      <c r="G70">
+        <v>120</v>
+      </c>
+      <c r="H70" t="s">
+        <v>524</v>
+      </c>
+      <c r="I70">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="71" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B71" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D71" t="s">
+        <v>261</v>
+      </c>
+      <c r="E71" t="s">
+        <v>84</v>
+      </c>
+      <c r="F71">
+        <v>64</v>
+      </c>
+      <c r="G71">
+        <v>256</v>
+      </c>
+      <c r="H71" t="s">
+        <v>524</v>
+      </c>
+      <c r="I71">
+        <v>1.0666666666666667</v>
+      </c>
+    </row>
+    <row r="72" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B72" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D72" t="s">
+        <v>297</v>
+      </c>
+      <c r="E72" t="s">
+        <v>121</v>
+      </c>
+      <c r="F72">
+        <v>400</v>
+      </c>
+      <c r="G72">
+        <v>800</v>
+      </c>
+      <c r="H72" t="s">
+        <v>524</v>
+      </c>
+      <c r="I72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B73" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C73" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D73" t="s">
+        <v>362</v>
+      </c>
+      <c r="E73" t="s">
+        <v>186</v>
+      </c>
+      <c r="F73">
+        <v>72</v>
+      </c>
+      <c r="G73">
+        <v>216</v>
+      </c>
+      <c r="H73" t="s">
+        <v>525</v>
+      </c>
+      <c r="I73">
+        <v>0.98181818181818181</v>
+      </c>
+    </row>
+    <row r="74" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B74" s="64">
+        <v>46203</v>
+      </c>
+      <c r="C74" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D74" t="s">
+        <v>361</v>
+      </c>
+      <c r="E74" t="s">
+        <v>185</v>
+      </c>
+      <c r="F74">
+        <v>72</v>
+      </c>
+      <c r="G74">
+        <v>216</v>
+      </c>
+      <c r="H74" t="s">
+        <v>525</v>
+      </c>
+      <c r="I74">
+        <v>0.98181818181818181</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>